<commit_message>
Updated Exercise 4A files
</commit_message>
<xml_diff>
--- a/Luis-Espinosa-Vilicana/lastname_Ex3A_tables.xlsx
+++ b/Luis-Espinosa-Vilicana/lastname_Ex3A_tables.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luise\Documents\DATA_labs\W2_Workshop\Luis-Espinosa-Vilicana\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{999AB378-5FF5-4D5A-B872-E0DAC54D860C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89129C9A-1D2E-4CE9-9262-EC5B599AE6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" activeTab="2" xr2:uid="{C4D3C96D-2B09-48A1-9CB6-1B41B37AD349}"/>
+    <workbookView xWindow="-19290" yWindow="4910" windowWidth="19380" windowHeight="10530" activeTab="2" xr2:uid="{C4D3C96D-2B09-48A1-9CB6-1B41B37AD349}"/>
   </bookViews>
   <sheets>
-    <sheet name="Customer Info" sheetId="1" r:id="rId1"/>
-    <sheet name="Pet Info" sheetId="2" r:id="rId2"/>
-    <sheet name="Services" sheetId="3" r:id="rId3"/>
+    <sheet name="customer_info" sheetId="1" r:id="rId1"/>
+    <sheet name="pet_info" sheetId="2" r:id="rId2"/>
+    <sheet name="services" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,51 +38,111 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
-  <si>
-    <t>Customer ID</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>Payment</t>
-  </si>
-  <si>
-    <t>Phone Number</t>
-  </si>
-  <si>
-    <t>Pet ID</t>
-  </si>
-  <si>
-    <t>Pet Name</t>
-  </si>
-  <si>
-    <t>Pet Breed</t>
-  </si>
-  <si>
-    <t>Pet Color</t>
-  </si>
-  <si>
-    <t>Session ID</t>
-  </si>
-  <si>
-    <t>Session Rate</t>
-  </si>
-  <si>
-    <t>Cost</t>
-  </si>
-  <si>
-    <t>Session Qty</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
+  <si>
+    <t>First_Name</t>
+  </si>
+  <si>
+    <t>Last_Name</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Zip_Code</t>
+  </si>
+  <si>
+    <t>Customer_ID</t>
+  </si>
+  <si>
+    <t>Street_Address</t>
+  </si>
+  <si>
+    <t>Payment_Type</t>
+  </si>
+  <si>
+    <t>Phone_Number</t>
+  </si>
+  <si>
+    <t>Created_At</t>
+  </si>
+  <si>
+    <t>Pet_ID</t>
+  </si>
+  <si>
+    <t>Pet_Name</t>
+  </si>
+  <si>
+    <t>Pet_Breed</t>
+  </si>
+  <si>
+    <t>Pet_Color</t>
+  </si>
+  <si>
+    <t>Special_Notes</t>
+  </si>
+  <si>
+    <t>Session_ID</t>
+  </si>
+  <si>
+    <t>Session_Rate</t>
+  </si>
+  <si>
+    <t>Total_Cost</t>
+  </si>
+  <si>
+    <t>Session_Qty</t>
+  </si>
+  <si>
+    <t>Service_Date</t>
+  </si>
+  <si>
+    <t>Payment_Status</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>123 Sesame St</t>
+  </si>
+  <si>
+    <t>San Francisco</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Sparky</t>
+  </si>
+  <si>
+    <t>Chihauha</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Paid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="mm\-dd\-yyyy\ hh:mm:ss"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -124,10 +184,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,41 +524,91 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D45BE82E-60BA-4685-B1F1-365B894F7AD3}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="11.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.36328125" customWidth="1"/>
+    <col min="3" max="3" width="5.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2">
+        <v>94110</v>
+      </c>
+      <c r="H2">
+        <v>1234567890</v>
+      </c>
+      <c r="I2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" s="3">
+        <v>46127.441608796296</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2CE3132-E88E-47BC-BFA4-23817FC1D356}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.6328125" bestFit="1" customWidth="1"/>
@@ -505,21 +617,44 @@
     <col min="5" max="5" width="8.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="C1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E1" t="s">
-        <v>8</v>
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -529,31 +664,69 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76FD25CE-2C0B-4F35-8787-57143E5CD674}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46127</v>
+      </c>
+      <c r="E2">
+        <v>15</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>